<commit_message>
Update models to FY2025A actuals, remove Q&A files
DKS LBO:
- LTM Revenue $13.0B → $13.44B, EBITDA $1.70B → $1.87B
- SOFR 4.5% → 3.7%; TLB rate 8.0% → 7.2%
- Returns: 30.4% IRR / 3.8x MOIC → 28.1% IRR / 3.5x MOIC
- Deal memo and build scripts updated throughout
- OUTPUT_PATH corrected to repo directory

AMD DCF:
- FY2025E → FY2025A with actual segment data ($34.6B total)
- DC +31.6%, Client +51.9%, Gaming +53.3%, Embedded -3.8% YoY
- Current price $120 → $200; PT $145 → $215
- Sensitivity tables fully recomputed from new FCF base

READMEs:
- Root README: updated returns/PT figures, removed Q&A mention
- dks-lbo/README: complete rewrite with current model numbers
- amd-dcf/README: new file with FY2025A actuals and thesis
- ferrari-dcf/README: removed references to non-existent build scripts

Cleanup:
- Deleted AMD, DKS, Ferrari interview Q&A .md files

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dks-lbo/DKS_LBO_Model.xlsx
+++ b/dks-lbo/DKS_LBO_Model.xlsx
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="B4" s="16" t="n">
-        <v>13000</v>
+        <v>13440</v>
       </c>
     </row>
     <row r="5">
@@ -920,7 +920,7 @@
         </is>
       </c>
       <c r="B5" s="16" t="n">
-        <v>1700</v>
+        <v>1870</v>
       </c>
     </row>
     <row r="6">
@@ -1125,7 +1125,7 @@
         </is>
       </c>
       <c r="B27" s="24" t="n">
-        <v>0.045</v>
+        <v>0.037</v>
       </c>
     </row>
     <row r="28">

</xml_diff>

<commit_message>
Add branded footer/header to all model outputs
Excel: thin branded footer row on every sheet ("Francisco Rodriguez | Financial Modeling Portfolio | github.com/Azyo1") — added to DKS and NAUT build scripts and regenerated xlsx files.

PDF: running page header on every page (name left, doc title right, thin rule) — added to DKS and NAUT memo scripts and regenerated pdf files. topMargin bumped to 0.75in to clear the header.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dks-lbo/DKS_LBO_Model.xlsx
+++ b/dks-lbo/DKS_LBO_Model.xlsx
@@ -25,7 +25,7 @@
     <numFmt numFmtId="164" formatCode="0.0&quot;x&quot;"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -90,6 +90,12 @@
       <i val="1"/>
       <color rgb="009E9E9E"/>
       <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="009E9E9E"/>
+      <sz val="7.5"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -186,7 +192,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -227,84 +233,87 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="3" fontId="12" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="13" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="13" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="13" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="3" fontId="13" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="14" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="12" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="13" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="15" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="16" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="15" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="16" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="16" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="14" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="14" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -673,7 +682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B3:F22"/>
+  <dimension ref="B3:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -856,13 +865,21 @@
         </is>
       </c>
     </row>
+    <row r="24" ht="12" customHeight="1">
+      <c r="B24" s="15" t="inlineStr">
+        <is>
+          <t>Francisco Rodriguez  |  Financial Modeling Portfolio  |  github.com/Azyo1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="15">
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="C18:F18"/>
     <mergeCell ref="B7:F7"/>
     <mergeCell ref="C17:F17"/>
     <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B24:F24"/>
     <mergeCell ref="B16:F16"/>
     <mergeCell ref="C20:F20"/>
     <mergeCell ref="B3:F3"/>
@@ -884,7 +901,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A3:G46"/>
+  <dimension ref="A3:G48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -904,106 +921,106 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>LTM Revenue ($M)</t>
         </is>
       </c>
-      <c r="B4" s="16" t="n">
+      <c r="B4" s="17" t="n">
         <v>13440</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>LTM EBITDA ($M)</t>
         </is>
       </c>
-      <c r="B5" s="16" t="n">
+      <c r="B5" s="17" t="n">
         <v>1870</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>LTM EBITDA Margin</t>
         </is>
       </c>
-      <c r="B6" s="17">
+      <c r="B6" s="18">
         <f>B5/B4</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>Entry EV / LTM EBITDA Multiple</t>
         </is>
       </c>
-      <c r="B7" s="18" t="n">
+      <c r="B7" s="19" t="n">
         <v>9</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>Transaction Enterprise Value ($M)</t>
         </is>
       </c>
-      <c r="B8" s="19">
+      <c r="B8" s="20">
         <f>B5*B7</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>Existing Net Debt at Close ($M)</t>
         </is>
       </c>
-      <c r="B9" s="16" t="n">
+      <c r="B9" s="17" t="n">
         <v>300</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>Transaction Equity Value ($M)</t>
         </is>
       </c>
-      <c r="B10" s="19">
+      <c r="B10" s="20">
         <f>B8-B9</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>Transaction Fees (% of TEV)</t>
         </is>
       </c>
-      <c r="B11" s="20" t="n">
+      <c r="B11" s="21" t="n">
         <v>0.02</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>Transaction Fees ($M)</t>
         </is>
       </c>
-      <c r="B12" s="19">
+      <c r="B12" s="20">
         <f>B8*B11</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="22" t="inlineStr">
         <is>
           <t>Total Uses ($M)</t>
         </is>
       </c>
-      <c r="B13" s="22">
+      <c r="B13" s="23">
         <f>B10+B12</f>
         <v/>
       </c>
@@ -1016,97 +1033,97 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="15" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>Term Loan B — Leverage Multiple (x LTM EBITDA)</t>
         </is>
       </c>
-      <c r="B16" s="18" t="n">
+      <c r="B16" s="19" t="n">
         <v>5.5</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="15" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>Term Loan B ($M)</t>
         </is>
       </c>
-      <c r="B17" s="19">
+      <c r="B17" s="20">
         <f>B5*B16</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="15" t="inlineStr">
+      <c r="A18" s="16" t="inlineStr">
         <is>
           <t>Revolving Credit Facility — Capacity ($M)</t>
         </is>
       </c>
-      <c r="B18" s="16" t="n">
+      <c r="B18" s="17" t="n">
         <v>750</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="15" t="inlineStr">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>Revolving Credit Facility — Drawn at Close ($M)</t>
         </is>
       </c>
-      <c r="B19" s="16" t="n">
+      <c r="B19" s="17" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="15" t="inlineStr">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>Total Debt at Close ($M)</t>
         </is>
       </c>
-      <c r="B20" s="19">
+      <c r="B20" s="20">
         <f>B17+B19</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="15" t="inlineStr">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>Sponsor Equity ($M)</t>
         </is>
       </c>
-      <c r="B21" s="19">
+      <c r="B21" s="20">
         <f>B13-B20</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="21" t="inlineStr">
+      <c r="A22" s="22" t="inlineStr">
         <is>
           <t>Total Sources ($M)</t>
         </is>
       </c>
-      <c r="B22" s="22">
+      <c r="B22" s="23">
         <f>B20+B21</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="15" t="inlineStr">
+      <c r="A23" s="16" t="inlineStr">
         <is>
           <t>Leverage at Close (x LTM EBITDA)</t>
         </is>
       </c>
-      <c r="B23" s="23">
+      <c r="B23" s="24">
         <f>B20/B5</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="15" t="inlineStr">
+      <c r="A24" s="16" t="inlineStr">
         <is>
           <t>Equity Contribution (%)</t>
         </is>
       </c>
-      <c r="B24" s="17">
+      <c r="B24" s="18">
         <f>B21/B13</f>
         <v/>
       </c>
@@ -1119,84 +1136,84 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="15" t="inlineStr">
+      <c r="A27" s="16" t="inlineStr">
         <is>
           <t>Base Rate (SOFR)</t>
         </is>
       </c>
-      <c r="B27" s="24" t="n">
+      <c r="B27" s="25" t="n">
         <v>0.037</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="15" t="inlineStr">
+      <c r="A28" s="16" t="inlineStr">
         <is>
           <t>Term Loan B — Credit Spread</t>
         </is>
       </c>
-      <c r="B28" s="24" t="n">
+      <c r="B28" s="25" t="n">
         <v>0.035</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="15" t="inlineStr">
+      <c r="A29" s="16" t="inlineStr">
         <is>
           <t>Term Loan B — All-In Interest Rate</t>
         </is>
       </c>
-      <c r="B29" s="25">
+      <c r="B29" s="26">
         <f>B27+B28</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="15" t="inlineStr">
+      <c r="A30" s="16" t="inlineStr">
         <is>
           <t>Term Loan B — Annual Amortization (%)</t>
         </is>
       </c>
-      <c r="B30" s="20" t="n">
+      <c r="B30" s="21" t="n">
         <v>0.01</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="15" t="inlineStr">
+      <c r="A31" s="16" t="inlineStr">
         <is>
           <t>Revolving Credit Facility — Credit Spread</t>
         </is>
       </c>
-      <c r="B31" s="24" t="n">
+      <c r="B31" s="25" t="n">
         <v>0.0275</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="15" t="inlineStr">
+      <c r="A32" s="16" t="inlineStr">
         <is>
           <t>Revolving Credit Facility — All-In Rate</t>
         </is>
       </c>
-      <c r="B32" s="25">
+      <c r="B32" s="26">
         <f>B27+B31</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="15" t="inlineStr">
+      <c r="A33" s="16" t="inlineStr">
         <is>
           <t>Undrawn Commitment Fee (%)</t>
         </is>
       </c>
-      <c r="B33" s="24" t="n">
+      <c r="B33" s="25" t="n">
         <v>0.00375</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="15" t="inlineStr">
+      <c r="A34" s="16" t="inlineStr">
         <is>
           <t>Cash Tax Rate</t>
         </is>
       </c>
-      <c r="B34" s="20" t="n">
+      <c r="B34" s="21" t="n">
         <v>0.25</v>
       </c>
     </row>
@@ -1206,140 +1223,140 @@
           <t>OPERATING ASSUMPTIONS</t>
         </is>
       </c>
-      <c r="B36" s="26" t="n"/>
-      <c r="C36" s="27" t="inlineStr">
+      <c r="B36" s="27" t="n"/>
+      <c r="C36" s="28" t="inlineStr">
         <is>
           <t>Year 1</t>
         </is>
       </c>
-      <c r="D36" s="27" t="inlineStr">
+      <c r="D36" s="28" t="inlineStr">
         <is>
           <t>Year 2</t>
         </is>
       </c>
-      <c r="E36" s="27" t="inlineStr">
+      <c r="E36" s="28" t="inlineStr">
         <is>
           <t>Year 3</t>
         </is>
       </c>
-      <c r="F36" s="27" t="inlineStr">
+      <c r="F36" s="28" t="inlineStr">
         <is>
           <t>Year 4</t>
         </is>
       </c>
-      <c r="G36" s="27" t="inlineStr">
+      <c r="G36" s="28" t="inlineStr">
         <is>
           <t>Year 5</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="15" t="inlineStr">
+      <c r="A37" s="16" t="inlineStr">
         <is>
           <t>Revenue Growth</t>
         </is>
       </c>
-      <c r="C37" s="20" t="n">
+      <c r="C37" s="21" t="n">
         <v>0.04</v>
       </c>
-      <c r="D37" s="20" t="n">
+      <c r="D37" s="21" t="n">
         <v>0.04</v>
       </c>
-      <c r="E37" s="20" t="n">
+      <c r="E37" s="21" t="n">
         <v>0.05</v>
       </c>
-      <c r="F37" s="20" t="n">
+      <c r="F37" s="21" t="n">
         <v>0.05</v>
       </c>
-      <c r="G37" s="20" t="n">
+      <c r="G37" s="21" t="n">
         <v>0.05</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="15" t="inlineStr">
+      <c r="A38" s="16" t="inlineStr">
         <is>
           <t>EBITDA Margin</t>
         </is>
       </c>
-      <c r="C38" s="20" t="n">
+      <c r="C38" s="21" t="n">
         <v>0.14</v>
       </c>
-      <c r="D38" s="20" t="n">
+      <c r="D38" s="21" t="n">
         <v>0.15</v>
       </c>
-      <c r="E38" s="20" t="n">
+      <c r="E38" s="21" t="n">
         <v>0.155</v>
       </c>
-      <c r="F38" s="20" t="n">
+      <c r="F38" s="21" t="n">
         <v>0.16</v>
       </c>
-      <c r="G38" s="20" t="n">
+      <c r="G38" s="21" t="n">
         <v>0.165</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="15" t="inlineStr">
+      <c r="A39" s="16" t="inlineStr">
         <is>
           <t>D&amp;A (% of Revenue)</t>
         </is>
       </c>
-      <c r="C39" s="20" t="n">
+      <c r="C39" s="21" t="n">
         <v>0.027</v>
       </c>
-      <c r="D39" s="20" t="n">
+      <c r="D39" s="21" t="n">
         <v>0.027</v>
       </c>
-      <c r="E39" s="20" t="n">
+      <c r="E39" s="21" t="n">
         <v>0.027</v>
       </c>
-      <c r="F39" s="20" t="n">
+      <c r="F39" s="21" t="n">
         <v>0.027</v>
       </c>
-      <c r="G39" s="20" t="n">
+      <c r="G39" s="21" t="n">
         <v>0.027</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="15" t="inlineStr">
+      <c r="A40" s="16" t="inlineStr">
         <is>
           <t>Capital Expenditures (% of Revenue)</t>
         </is>
       </c>
-      <c r="C40" s="20" t="n">
+      <c r="C40" s="21" t="n">
         <v>0.035</v>
       </c>
-      <c r="D40" s="20" t="n">
+      <c r="D40" s="21" t="n">
         <v>0.035</v>
       </c>
-      <c r="E40" s="20" t="n">
+      <c r="E40" s="21" t="n">
         <v>0.035</v>
       </c>
-      <c r="F40" s="20" t="n">
+      <c r="F40" s="21" t="n">
         <v>0.035</v>
       </c>
-      <c r="G40" s="20" t="n">
+      <c r="G40" s="21" t="n">
         <v>0.035</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="15" t="inlineStr">
+      <c r="A41" s="16" t="inlineStr">
         <is>
           <t>Change in NWC (% of Δ Revenue)</t>
         </is>
       </c>
-      <c r="C41" s="20" t="n">
+      <c r="C41" s="21" t="n">
         <v>0.05</v>
       </c>
-      <c r="D41" s="20" t="n">
+      <c r="D41" s="21" t="n">
         <v>0.05</v>
       </c>
-      <c r="E41" s="20" t="n">
+      <c r="E41" s="21" t="n">
         <v>0.05</v>
       </c>
-      <c r="F41" s="20" t="n">
+      <c r="F41" s="21" t="n">
         <v>0.05</v>
       </c>
-      <c r="G41" s="20" t="n">
+      <c r="G41" s="21" t="n">
         <v>0.05</v>
       </c>
     </row>
@@ -1351,41 +1368,49 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="15" t="inlineStr">
+      <c r="A44" s="16" t="inlineStr">
         <is>
           <t>Exit Year</t>
         </is>
       </c>
-      <c r="B44" s="28" t="n">
+      <c r="B44" s="29" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="15" t="inlineStr">
+      <c r="A45" s="16" t="inlineStr">
         <is>
           <t>Exit EV / EBITDA Multiple</t>
         </is>
       </c>
-      <c r="B45" s="18" t="n">
+      <c r="B45" s="19" t="n">
         <v>10.5</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="15" t="inlineStr">
+      <c r="A46" s="16" t="inlineStr">
         <is>
           <t>Exit Transaction Fees (% of TEV)</t>
         </is>
       </c>
-      <c r="B46" s="20" t="n">
+      <c r="B46" s="21" t="n">
         <v>0.01</v>
       </c>
     </row>
+    <row r="48" ht="12" customHeight="1">
+      <c r="B48" s="15" t="inlineStr">
+        <is>
+          <t>Francisco Rodriguez  |  Financial Modeling Portfolio  |  github.com/Azyo1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="A15:G15"/>
     <mergeCell ref="A43:G43"/>
-    <mergeCell ref="A26:G26"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="B48:G48"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1398,7 +1423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -1411,40 +1436,40 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="29" t="inlineStr">
+      <c r="A1" s="30" t="inlineStr">
         <is>
           <t>Dick's Sporting Goods — Operating Model</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="27" t="inlineStr"/>
-      <c r="B3" s="27" t="inlineStr">
+      <c r="A3" s="28" t="inlineStr"/>
+      <c r="B3" s="28" t="inlineStr">
         <is>
           <t>LTM</t>
         </is>
       </c>
-      <c r="C3" s="27" t="inlineStr">
+      <c r="C3" s="28" t="inlineStr">
         <is>
           <t>Year 1</t>
         </is>
       </c>
-      <c r="D3" s="27" t="inlineStr">
+      <c r="D3" s="28" t="inlineStr">
         <is>
           <t>Year 2</t>
         </is>
       </c>
-      <c r="E3" s="27" t="inlineStr">
+      <c r="E3" s="28" t="inlineStr">
         <is>
           <t>Year 3</t>
         </is>
       </c>
-      <c r="F3" s="27" t="inlineStr">
+      <c r="F3" s="28" t="inlineStr">
         <is>
           <t>Year 4</t>
         </is>
       </c>
-      <c r="G3" s="27" t="inlineStr">
+      <c r="G3" s="28" t="inlineStr">
         <is>
           <t>Year 5</t>
         </is>
@@ -1458,390 +1483,390 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="30" t="inlineStr">
+      <c r="A5" s="31" t="inlineStr">
         <is>
           <t>Revenue</t>
         </is>
       </c>
-      <c r="B5" s="31">
+      <c r="B5" s="32">
         <f>'Assumptions'!B4</f>
         <v/>
       </c>
-      <c r="C5" s="19">
+      <c r="C5" s="20">
         <f>B5*(1+'Assumptions'!C37)</f>
         <v/>
       </c>
-      <c r="D5" s="19">
+      <c r="D5" s="20">
         <f>C5*(1+'Assumptions'!D37)</f>
         <v/>
       </c>
-      <c r="E5" s="19">
+      <c r="E5" s="20">
         <f>D5*(1+'Assumptions'!E37)</f>
         <v/>
       </c>
-      <c r="F5" s="19">
+      <c r="F5" s="20">
         <f>E5*(1+'Assumptions'!F37)</f>
         <v/>
       </c>
-      <c r="G5" s="19">
+      <c r="G5" s="20">
         <f>F5*(1+'Assumptions'!G37)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="32" t="inlineStr">
+      <c r="A6" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Revenue Growth %</t>
         </is>
       </c>
-      <c r="B6" s="33" t="inlineStr">
+      <c r="B6" s="34" t="inlineStr">
         <is>
           <t>LTM</t>
         </is>
       </c>
-      <c r="C6" s="17">
+      <c r="C6" s="18">
         <f>C5/B5-1</f>
         <v/>
       </c>
-      <c r="D6" s="17">
+      <c r="D6" s="18">
         <f>D5/C5-1</f>
         <v/>
       </c>
-      <c r="E6" s="17">
+      <c r="E6" s="18">
         <f>E5/D5-1</f>
         <v/>
       </c>
-      <c r="F6" s="17">
+      <c r="F6" s="18">
         <f>F5/E5-1</f>
         <v/>
       </c>
-      <c r="G6" s="17">
+      <c r="G6" s="18">
         <f>G5/F5-1</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="30" t="inlineStr">
+      <c r="A8" s="31" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="B8" s="31">
+      <c r="B8" s="32">
         <f>'Assumptions'!B5</f>
         <v/>
       </c>
-      <c r="C8" s="19">
+      <c r="C8" s="20">
         <f>C5*'Assumptions'!C38</f>
         <v/>
       </c>
-      <c r="D8" s="19">
+      <c r="D8" s="20">
         <f>D5*'Assumptions'!D38</f>
         <v/>
       </c>
-      <c r="E8" s="19">
+      <c r="E8" s="20">
         <f>E5*'Assumptions'!E38</f>
         <v/>
       </c>
-      <c r="F8" s="19">
+      <c r="F8" s="20">
         <f>F5*'Assumptions'!F38</f>
         <v/>
       </c>
-      <c r="G8" s="19">
+      <c r="G8" s="20">
         <f>G5*'Assumptions'!G38</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="32" t="inlineStr">
+      <c r="A9" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  EBITDA Margin %</t>
         </is>
       </c>
-      <c r="B9" s="17">
+      <c r="B9" s="18">
         <f>B8/B5</f>
         <v/>
       </c>
-      <c r="C9" s="17">
+      <c r="C9" s="18">
         <f>C8/C5</f>
         <v/>
       </c>
-      <c r="D9" s="17">
+      <c r="D9" s="18">
         <f>D8/D5</f>
         <v/>
       </c>
-      <c r="E9" s="17">
+      <c r="E9" s="18">
         <f>E8/E5</f>
         <v/>
       </c>
-      <c r="F9" s="17">
+      <c r="F9" s="18">
         <f>F8/F5</f>
         <v/>
       </c>
-      <c r="G9" s="17">
+      <c r="G9" s="18">
         <f>G8/G5</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="32" t="inlineStr">
+      <c r="A11" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Depreciation &amp; Amortization</t>
         </is>
       </c>
-      <c r="B11" s="19">
+      <c r="B11" s="20">
         <f>B5*'Assumptions'!C39</f>
         <v/>
       </c>
-      <c r="C11" s="19">
+      <c r="C11" s="20">
         <f>C5*'Assumptions'!C39</f>
         <v/>
       </c>
-      <c r="D11" s="19">
+      <c r="D11" s="20">
         <f>D5*'Assumptions'!D39</f>
         <v/>
       </c>
-      <c r="E11" s="19">
+      <c r="E11" s="20">
         <f>E5*'Assumptions'!E39</f>
         <v/>
       </c>
-      <c r="F11" s="19">
+      <c r="F11" s="20">
         <f>F5*'Assumptions'!F39</f>
         <v/>
       </c>
-      <c r="G11" s="19">
+      <c r="G11" s="20">
         <f>G5*'Assumptions'!G39</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="30" t="inlineStr">
+      <c r="A12" s="31" t="inlineStr">
         <is>
           <t>EBIT</t>
         </is>
       </c>
-      <c r="B12" s="19">
+      <c r="B12" s="20">
         <f>B8-B11</f>
         <v/>
       </c>
-      <c r="C12" s="19">
+      <c r="C12" s="20">
         <f>C8-C11</f>
         <v/>
       </c>
-      <c r="D12" s="19">
+      <c r="D12" s="20">
         <f>D8-D11</f>
         <v/>
       </c>
-      <c r="E12" s="19">
+      <c r="E12" s="20">
         <f>E8-E11</f>
         <v/>
       </c>
-      <c r="F12" s="19">
+      <c r="F12" s="20">
         <f>F8-F11</f>
         <v/>
       </c>
-      <c r="G12" s="19">
+      <c r="G12" s="20">
         <f>G8-G11</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="32" t="inlineStr">
+      <c r="A13" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  EBIT Margin %</t>
         </is>
       </c>
-      <c r="B13" s="17">
+      <c r="B13" s="18">
         <f>B12/B5</f>
         <v/>
       </c>
-      <c r="C13" s="17">
+      <c r="C13" s="18">
         <f>C12/C5</f>
         <v/>
       </c>
-      <c r="D13" s="17">
+      <c r="D13" s="18">
         <f>D12/D5</f>
         <v/>
       </c>
-      <c r="E13" s="17">
+      <c r="E13" s="18">
         <f>E12/E5</f>
         <v/>
       </c>
-      <c r="F13" s="17">
+      <c r="F13" s="18">
         <f>F12/F5</f>
         <v/>
       </c>
-      <c r="G13" s="17">
+      <c r="G13" s="18">
         <f>G12/G5</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="32" t="inlineStr">
+      <c r="A15" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Less: Interest Expense — TLB</t>
         </is>
       </c>
-      <c r="B15" s="19" t="n">
+      <c r="B15" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="C15" s="31">
+      <c r="C15" s="32">
         <f>'Debt Schedule'!C10</f>
         <v/>
       </c>
-      <c r="D15" s="31">
+      <c r="D15" s="32">
         <f>'Debt Schedule'!D10</f>
         <v/>
       </c>
-      <c r="E15" s="31">
+      <c r="E15" s="32">
         <f>'Debt Schedule'!E10</f>
         <v/>
       </c>
-      <c r="F15" s="31">
+      <c r="F15" s="32">
         <f>'Debt Schedule'!F10</f>
         <v/>
       </c>
-      <c r="G15" s="31">
+      <c r="G15" s="32">
         <f>'Debt Schedule'!G10</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="32" t="inlineStr">
+      <c r="A16" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Less: Interest Expense — Revolver</t>
         </is>
       </c>
-      <c r="B16" s="19" t="n">
+      <c r="B16" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="C16" s="31">
+      <c r="C16" s="32">
         <f>'Debt Schedule'!C17</f>
         <v/>
       </c>
-      <c r="D16" s="31">
+      <c r="D16" s="32">
         <f>'Debt Schedule'!D17</f>
         <v/>
       </c>
-      <c r="E16" s="31">
+      <c r="E16" s="32">
         <f>'Debt Schedule'!E17</f>
         <v/>
       </c>
-      <c r="F16" s="31">
+      <c r="F16" s="32">
         <f>'Debt Schedule'!F17</f>
         <v/>
       </c>
-      <c r="G16" s="31">
+      <c r="G16" s="32">
         <f>'Debt Schedule'!G17</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="30" t="inlineStr">
+      <c r="A17" s="31" t="inlineStr">
         <is>
           <t>Total Interest Expense</t>
         </is>
       </c>
-      <c r="B17" s="19" t="n">
+      <c r="B17" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="C17" s="19">
+      <c r="C17" s="20">
         <f>C15+C16</f>
         <v/>
       </c>
-      <c r="D17" s="19">
+      <c r="D17" s="20">
         <f>D15+D16</f>
         <v/>
       </c>
-      <c r="E17" s="19">
+      <c r="E17" s="20">
         <f>E15+E16</f>
         <v/>
       </c>
-      <c r="F17" s="19">
+      <c r="F17" s="20">
         <f>F15+F16</f>
         <v/>
       </c>
-      <c r="G17" s="19">
+      <c r="G17" s="20">
         <f>G15+G16</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="30" t="inlineStr">
+      <c r="A19" s="31" t="inlineStr">
         <is>
           <t>EBT (Earnings Before Tax)</t>
         </is>
       </c>
-      <c r="C19" s="19">
+      <c r="C19" s="20">
         <f>MAX(0,C12-C17)</f>
         <v/>
       </c>
-      <c r="D19" s="19">
+      <c r="D19" s="20">
         <f>MAX(0,D12-D17)</f>
         <v/>
       </c>
-      <c r="E19" s="19">
+      <c r="E19" s="20">
         <f>MAX(0,E12-E17)</f>
         <v/>
       </c>
-      <c r="F19" s="19">
+      <c r="F19" s="20">
         <f>MAX(0,F12-F17)</f>
         <v/>
       </c>
-      <c r="G19" s="19">
+      <c r="G19" s="20">
         <f>MAX(0,G12-G17)</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="32" t="inlineStr">
+      <c r="A20" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Less: Income Tax Expense</t>
         </is>
       </c>
-      <c r="C20" s="19">
+      <c r="C20" s="20">
         <f>MAX(0,C19)*'Assumptions'!B34</f>
         <v/>
       </c>
-      <c r="D20" s="19">
+      <c r="D20" s="20">
         <f>MAX(0,D19)*'Assumptions'!B34</f>
         <v/>
       </c>
-      <c r="E20" s="19">
+      <c r="E20" s="20">
         <f>MAX(0,E19)*'Assumptions'!B34</f>
         <v/>
       </c>
-      <c r="F20" s="19">
+      <c r="F20" s="20">
         <f>MAX(0,F19)*'Assumptions'!B34</f>
         <v/>
       </c>
-      <c r="G20" s="19">
+      <c r="G20" s="20">
         <f>MAX(0,G19)*'Assumptions'!B34</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="30" t="inlineStr">
+      <c r="A21" s="31" t="inlineStr">
         <is>
           <t>Net Income</t>
         </is>
       </c>
-      <c r="C21" s="22">
+      <c r="C21" s="23">
         <f>C19-C20</f>
         <v/>
       </c>
-      <c r="D21" s="22">
+      <c r="D21" s="23">
         <f>D19-D20</f>
         <v/>
       </c>
-      <c r="E21" s="22">
+      <c r="E21" s="23">
         <f>E19-E20</f>
         <v/>
       </c>
-      <c r="F21" s="22">
+      <c r="F21" s="23">
         <f>F19-F20</f>
         <v/>
       </c>
-      <c r="G21" s="22">
+      <c r="G21" s="23">
         <f>G19-G20</f>
         <v/>
       </c>
@@ -1854,223 +1879,231 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="32" t="inlineStr">
+      <c r="A24" s="33" t="inlineStr">
         <is>
           <t>EBITDA</t>
         </is>
       </c>
-      <c r="C24" s="19">
+      <c r="C24" s="20">
         <f>C8</f>
         <v/>
       </c>
-      <c r="D24" s="19">
+      <c r="D24" s="20">
         <f>D8</f>
         <v/>
       </c>
-      <c r="E24" s="19">
+      <c r="E24" s="20">
         <f>E8</f>
         <v/>
       </c>
-      <c r="F24" s="19">
+      <c r="F24" s="20">
         <f>F8</f>
         <v/>
       </c>
-      <c r="G24" s="19">
+      <c r="G24" s="20">
         <f>G8</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="32" t="inlineStr">
+      <c r="A25" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Less: Cash Taxes</t>
         </is>
       </c>
-      <c r="C25" s="19">
+      <c r="C25" s="20">
         <f>-MAX(0,C12-C17)*'Assumptions'!B34</f>
         <v/>
       </c>
-      <c r="D25" s="19">
+      <c r="D25" s="20">
         <f>-MAX(0,D12-D17)*'Assumptions'!B34</f>
         <v/>
       </c>
-      <c r="E25" s="19">
+      <c r="E25" s="20">
         <f>-MAX(0,E12-E17)*'Assumptions'!B34</f>
         <v/>
       </c>
-      <c r="F25" s="19">
+      <c r="F25" s="20">
         <f>-MAX(0,F12-F17)*'Assumptions'!B34</f>
         <v/>
       </c>
-      <c r="G25" s="19">
+      <c r="G25" s="20">
         <f>-MAX(0,G12-G17)*'Assumptions'!B34</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="32" t="inlineStr">
+      <c r="A26" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Less: Capital Expenditures</t>
         </is>
       </c>
-      <c r="C26" s="19">
+      <c r="C26" s="20">
         <f>-C5*'Assumptions'!C40</f>
         <v/>
       </c>
-      <c r="D26" s="19">
+      <c r="D26" s="20">
         <f>-D5*'Assumptions'!D40</f>
         <v/>
       </c>
-      <c r="E26" s="19">
+      <c r="E26" s="20">
         <f>-E5*'Assumptions'!E40</f>
         <v/>
       </c>
-      <c r="F26" s="19">
+      <c r="F26" s="20">
         <f>-F5*'Assumptions'!F40</f>
         <v/>
       </c>
-      <c r="G26" s="19">
+      <c r="G26" s="20">
         <f>-G5*'Assumptions'!G40</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="32" t="inlineStr">
+      <c r="A27" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Less: Change in Net Working Capital</t>
         </is>
       </c>
-      <c r="C27" s="19">
+      <c r="C27" s="20">
         <f>-(C5-B5)*'Assumptions'!C41</f>
         <v/>
       </c>
-      <c r="D27" s="19">
+      <c r="D27" s="20">
         <f>-(D5-C5)*'Assumptions'!D41</f>
         <v/>
       </c>
-      <c r="E27" s="19">
+      <c r="E27" s="20">
         <f>-(E5-D5)*'Assumptions'!E41</f>
         <v/>
       </c>
-      <c r="F27" s="19">
+      <c r="F27" s="20">
         <f>-(F5-E5)*'Assumptions'!F41</f>
         <v/>
       </c>
-      <c r="G27" s="19">
+      <c r="G27" s="20">
         <f>-(G5-F5)*'Assumptions'!G41</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="30" t="inlineStr">
+      <c r="A28" s="31" t="inlineStr">
         <is>
           <t>Unlevered Free Cash Flow</t>
         </is>
       </c>
-      <c r="C28" s="22">
+      <c r="C28" s="23">
         <f>C24+C25+C26+C27</f>
         <v/>
       </c>
-      <c r="D28" s="22">
+      <c r="D28" s="23">
         <f>D24+D25+D26+D27</f>
         <v/>
       </c>
-      <c r="E28" s="22">
+      <c r="E28" s="23">
         <f>E24+E25+E26+E27</f>
         <v/>
       </c>
-      <c r="F28" s="22">
+      <c r="F28" s="23">
         <f>F24+F25+F26+F27</f>
         <v/>
       </c>
-      <c r="G28" s="22">
+      <c r="G28" s="23">
         <f>G24+G25+G26+G27</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="32" t="inlineStr">
+      <c r="A30" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Less: Total Interest Expense</t>
         </is>
       </c>
-      <c r="C30" s="19">
+      <c r="C30" s="20">
         <f>-C17</f>
         <v/>
       </c>
-      <c r="D30" s="19">
+      <c r="D30" s="20">
         <f>-D17</f>
         <v/>
       </c>
-      <c r="E30" s="19">
+      <c r="E30" s="20">
         <f>-E17</f>
         <v/>
       </c>
-      <c r="F30" s="19">
+      <c r="F30" s="20">
         <f>-F17</f>
         <v/>
       </c>
-      <c r="G30" s="19">
+      <c r="G30" s="20">
         <f>-G17</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="32" t="inlineStr">
+      <c r="A31" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Less: Mandatory TLB Amortization</t>
         </is>
       </c>
-      <c r="C31" s="31">
+      <c r="C31" s="32">
         <f>'Debt Schedule'!C6</f>
         <v/>
       </c>
-      <c r="D31" s="31">
+      <c r="D31" s="32">
         <f>'Debt Schedule'!D6</f>
         <v/>
       </c>
-      <c r="E31" s="31">
+      <c r="E31" s="32">
         <f>'Debt Schedule'!E6</f>
         <v/>
       </c>
-      <c r="F31" s="31">
+      <c r="F31" s="32">
         <f>'Debt Schedule'!F6</f>
         <v/>
       </c>
-      <c r="G31" s="31">
+      <c r="G31" s="32">
         <f>'Debt Schedule'!G6</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="30" t="inlineStr">
+      <c r="A32" s="31" t="inlineStr">
         <is>
           <t>Levered Free Cash Flow</t>
         </is>
       </c>
-      <c r="C32" s="22">
+      <c r="C32" s="23">
         <f>C28+C30+C31</f>
         <v/>
       </c>
-      <c r="D32" s="22">
+      <c r="D32" s="23">
         <f>D28+D30+D31</f>
         <v/>
       </c>
-      <c r="E32" s="22">
+      <c r="E32" s="23">
         <f>E28+E30+E31</f>
         <v/>
       </c>
-      <c r="F32" s="22">
+      <c r="F32" s="23">
         <f>F28+F30+F31</f>
         <v/>
       </c>
-      <c r="G32" s="22">
+      <c r="G32" s="23">
         <f>G28+G30+G31</f>
         <v/>
       </c>
     </row>
+    <row r="34" ht="12" customHeight="1">
+      <c r="B34" s="15" t="inlineStr">
+        <is>
+          <t>Francisco Rodriguez  |  Financial Modeling Portfolio  |  github.com/Azyo1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
+    <mergeCell ref="B34:G34"/>
     <mergeCell ref="A23:G23"/>
     <mergeCell ref="A4:G4"/>
   </mergeCells>
@@ -2085,7 +2118,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -2098,35 +2131,35 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="29" t="inlineStr">
+      <c r="A1" s="30" t="inlineStr">
         <is>
           <t>Dick's Sporting Goods — Debt Schedule</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="27" t="inlineStr"/>
-      <c r="C3" s="27" t="inlineStr">
+      <c r="A3" s="28" t="inlineStr"/>
+      <c r="C3" s="28" t="inlineStr">
         <is>
           <t>Year 1</t>
         </is>
       </c>
-      <c r="D3" s="27" t="inlineStr">
+      <c r="D3" s="28" t="inlineStr">
         <is>
           <t>Year 2</t>
         </is>
       </c>
-      <c r="E3" s="27" t="inlineStr">
+      <c r="E3" s="28" t="inlineStr">
         <is>
           <t>Year 3</t>
         </is>
       </c>
-      <c r="F3" s="27" t="inlineStr">
+      <c r="F3" s="28" t="inlineStr">
         <is>
           <t>Year 4</t>
         </is>
       </c>
-      <c r="G3" s="27" t="inlineStr">
+      <c r="G3" s="28" t="inlineStr">
         <is>
           <t>Year 5</t>
         </is>
@@ -2140,163 +2173,163 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="32" t="inlineStr">
+      <c r="A5" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Beginning Balance</t>
         </is>
       </c>
-      <c r="C5" s="31">
+      <c r="C5" s="32">
         <f>'Assumptions'!B17</f>
         <v/>
       </c>
-      <c r="D5" s="19">
+      <c r="D5" s="20">
         <f>C8</f>
         <v/>
       </c>
-      <c r="E5" s="19">
+      <c r="E5" s="20">
         <f>D8</f>
         <v/>
       </c>
-      <c r="F5" s="19">
+      <c r="F5" s="20">
         <f>E8</f>
         <v/>
       </c>
-      <c r="G5" s="19">
+      <c r="G5" s="20">
         <f>F8</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="32" t="inlineStr">
+      <c r="A6" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Less: Mandatory Amortization</t>
         </is>
       </c>
-      <c r="C6" s="19">
+      <c r="C6" s="20">
         <f>-'Assumptions'!B17*'Assumptions'!B30</f>
         <v/>
       </c>
-      <c r="D6" s="19">
+      <c r="D6" s="20">
         <f>-'Assumptions'!B17*'Assumptions'!B30</f>
         <v/>
       </c>
-      <c r="E6" s="19">
+      <c r="E6" s="20">
         <f>-'Assumptions'!B17*'Assumptions'!B30</f>
         <v/>
       </c>
-      <c r="F6" s="19">
+      <c r="F6" s="20">
         <f>-'Assumptions'!B17*'Assumptions'!B30</f>
         <v/>
       </c>
-      <c r="G6" s="19">
+      <c r="G6" s="20">
         <f>-'Assumptions'!B17*'Assumptions'!B30</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="32" t="inlineStr">
+      <c r="A7" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Less: Cash Sweep</t>
         </is>
       </c>
-      <c r="C7" s="19">
+      <c r="C7" s="20">
         <f>-MAX(0,'Operating Model'!C32)</f>
         <v/>
       </c>
-      <c r="D7" s="19">
+      <c r="D7" s="20">
         <f>-MAX(0,'Operating Model'!D32)</f>
         <v/>
       </c>
-      <c r="E7" s="19">
+      <c r="E7" s="20">
         <f>-MAX(0,'Operating Model'!E32)</f>
         <v/>
       </c>
-      <c r="F7" s="19">
+      <c r="F7" s="20">
         <f>-MAX(0,'Operating Model'!F32)</f>
         <v/>
       </c>
-      <c r="G7" s="19">
+      <c r="G7" s="20">
         <f>-MAX(0,'Operating Model'!G32)</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="30" t="inlineStr">
+      <c r="A8" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  Ending Balance</t>
         </is>
       </c>
-      <c r="C8" s="22">
+      <c r="C8" s="23">
         <f>MAX(0,C5+C6+C7)</f>
         <v/>
       </c>
-      <c r="D8" s="22">
+      <c r="D8" s="23">
         <f>MAX(0,D5+D6+D7)</f>
         <v/>
       </c>
-      <c r="E8" s="22">
+      <c r="E8" s="23">
         <f>MAX(0,E5+E6+E7)</f>
         <v/>
       </c>
-      <c r="F8" s="22">
+      <c r="F8" s="23">
         <f>MAX(0,F5+F6+F7)</f>
         <v/>
       </c>
-      <c r="G8" s="22">
+      <c r="G8" s="23">
         <f>MAX(0,G5+G6+G7)</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="32" t="inlineStr">
+      <c r="A9" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Interest Rate</t>
         </is>
       </c>
-      <c r="C9" s="34">
+      <c r="C9" s="35">
         <f>'Assumptions'!B29</f>
         <v/>
       </c>
-      <c r="D9" s="34">
+      <c r="D9" s="35">
         <f>'Assumptions'!B29</f>
         <v/>
       </c>
-      <c r="E9" s="34">
+      <c r="E9" s="35">
         <f>'Assumptions'!B29</f>
         <v/>
       </c>
-      <c r="F9" s="34">
+      <c r="F9" s="35">
         <f>'Assumptions'!B29</f>
         <v/>
       </c>
-      <c r="G9" s="34">
+      <c r="G9" s="35">
         <f>'Assumptions'!B29</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="30" t="inlineStr">
+      <c r="A10" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  Interest Expense — TLB</t>
         </is>
       </c>
-      <c r="C10" s="22">
+      <c r="C10" s="23">
         <f>C5*C9</f>
         <v/>
       </c>
-      <c r="D10" s="22">
+      <c r="D10" s="23">
         <f>D5*D9</f>
         <v/>
       </c>
-      <c r="E10" s="22">
+      <c r="E10" s="23">
         <f>E5*E9</f>
         <v/>
       </c>
-      <c r="F10" s="22">
+      <c r="F10" s="23">
         <f>F5*F9</f>
         <v/>
       </c>
-      <c r="G10" s="22">
+      <c r="G10" s="23">
         <f>G5*G9</f>
         <v/>
       </c>
@@ -2309,136 +2342,136 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="32" t="inlineStr">
+      <c r="A13" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Beginning Balance</t>
         </is>
       </c>
-      <c r="C13" s="19">
+      <c r="C13" s="20">
         <f>0</f>
         <v/>
       </c>
-      <c r="D13" s="19">
+      <c r="D13" s="20">
         <f>0</f>
         <v/>
       </c>
-      <c r="E13" s="19">
+      <c r="E13" s="20">
         <f>0</f>
         <v/>
       </c>
-      <c r="F13" s="19">
+      <c r="F13" s="20">
         <f>0</f>
         <v/>
       </c>
-      <c r="G13" s="19">
+      <c r="G13" s="20">
         <f>0</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="32" t="inlineStr">
+      <c r="A14" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Draw / (Repayment)</t>
         </is>
       </c>
-      <c r="C14" s="19">
+      <c r="C14" s="20">
         <f>0</f>
         <v/>
       </c>
-      <c r="D14" s="19">
+      <c r="D14" s="20">
         <f>0</f>
         <v/>
       </c>
-      <c r="E14" s="19">
+      <c r="E14" s="20">
         <f>0</f>
         <v/>
       </c>
-      <c r="F14" s="19">
+      <c r="F14" s="20">
         <f>0</f>
         <v/>
       </c>
-      <c r="G14" s="19">
+      <c r="G14" s="20">
         <f>0</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="30" t="inlineStr">
+      <c r="A15" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  Ending Balance</t>
         </is>
       </c>
-      <c r="C15" s="22">
+      <c r="C15" s="23">
         <f>C13+C14</f>
         <v/>
       </c>
-      <c r="D15" s="22">
+      <c r="D15" s="23">
         <f>D13+D14</f>
         <v/>
       </c>
-      <c r="E15" s="22">
+      <c r="E15" s="23">
         <f>E13+E14</f>
         <v/>
       </c>
-      <c r="F15" s="22">
+      <c r="F15" s="23">
         <f>F13+F14</f>
         <v/>
       </c>
-      <c r="G15" s="22">
+      <c r="G15" s="23">
         <f>G13+G14</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="32" t="inlineStr">
+      <c r="A16" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Interest Rate (All-In)</t>
         </is>
       </c>
-      <c r="C16" s="34">
+      <c r="C16" s="35">
         <f>'Assumptions'!B32</f>
         <v/>
       </c>
-      <c r="D16" s="34">
+      <c r="D16" s="35">
         <f>'Assumptions'!B32</f>
         <v/>
       </c>
-      <c r="E16" s="34">
+      <c r="E16" s="35">
         <f>'Assumptions'!B32</f>
         <v/>
       </c>
-      <c r="F16" s="34">
+      <c r="F16" s="35">
         <f>'Assumptions'!B32</f>
         <v/>
       </c>
-      <c r="G16" s="34">
+      <c r="G16" s="35">
         <f>'Assumptions'!B32</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="30" t="inlineStr">
+      <c r="A17" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  Interest Expense — Revolver (Commitment Fee)</t>
         </is>
       </c>
-      <c r="C17" s="22">
+      <c r="C17" s="23">
         <f>'Assumptions'!B18*'Assumptions'!B33</f>
         <v/>
       </c>
-      <c r="D17" s="22">
+      <c r="D17" s="23">
         <f>'Assumptions'!B18*'Assumptions'!B33</f>
         <v/>
       </c>
-      <c r="E17" s="22">
+      <c r="E17" s="23">
         <f>'Assumptions'!B18*'Assumptions'!B33</f>
         <v/>
       </c>
-      <c r="F17" s="22">
+      <c r="F17" s="23">
         <f>'Assumptions'!B18*'Assumptions'!B33</f>
         <v/>
       </c>
-      <c r="G17" s="22">
+      <c r="G17" s="23">
         <f>'Assumptions'!B18*'Assumptions'!B33</f>
         <v/>
       </c>
@@ -2451,116 +2484,124 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="32" t="inlineStr">
+      <c r="A20" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Total Debt — Beginning</t>
         </is>
       </c>
-      <c r="C20" s="19">
+      <c r="C20" s="20">
         <f>C5+C13</f>
         <v/>
       </c>
-      <c r="D20" s="19">
+      <c r="D20" s="20">
         <f>D5+D13</f>
         <v/>
       </c>
-      <c r="E20" s="19">
+      <c r="E20" s="20">
         <f>E5+E13</f>
         <v/>
       </c>
-      <c r="F20" s="19">
+      <c r="F20" s="20">
         <f>F5+F13</f>
         <v/>
       </c>
-      <c r="G20" s="19">
+      <c r="G20" s="20">
         <f>G5+G13</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="30" t="inlineStr">
+      <c r="A21" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  Total Debt — Ending</t>
         </is>
       </c>
-      <c r="C21" s="22">
+      <c r="C21" s="23">
         <f>C8+C15</f>
         <v/>
       </c>
-      <c r="D21" s="22">
+      <c r="D21" s="23">
         <f>D8+D15</f>
         <v/>
       </c>
-      <c r="E21" s="22">
+      <c r="E21" s="23">
         <f>E8+E15</f>
         <v/>
       </c>
-      <c r="F21" s="22">
+      <c r="F21" s="23">
         <f>F8+F15</f>
         <v/>
       </c>
-      <c r="G21" s="22">
+      <c r="G21" s="23">
         <f>G8+G15</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="32" t="inlineStr">
+      <c r="A22" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Total Net Debt at Exit</t>
         </is>
       </c>
-      <c r="C22" s="19">
+      <c r="C22" s="20">
         <f>C21</f>
         <v/>
       </c>
-      <c r="D22" s="19">
+      <c r="D22" s="20">
         <f>D21</f>
         <v/>
       </c>
-      <c r="E22" s="19">
+      <c r="E22" s="20">
         <f>E21</f>
         <v/>
       </c>
-      <c r="F22" s="19">
+      <c r="F22" s="20">
         <f>F21</f>
         <v/>
       </c>
-      <c r="G22" s="19">
+      <c r="G22" s="20">
         <f>G21</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="32" t="inlineStr">
+      <c r="A23" s="33" t="inlineStr">
         <is>
           <t xml:space="preserve">  Leverage at Exit (x EBITDA)</t>
         </is>
       </c>
-      <c r="C23" s="23">
+      <c r="C23" s="24">
         <f>C21/'Operating Model'!C8</f>
         <v/>
       </c>
-      <c r="D23" s="23">
+      <c r="D23" s="24">
         <f>D21/'Operating Model'!D8</f>
         <v/>
       </c>
-      <c r="E23" s="23">
+      <c r="E23" s="24">
         <f>E21/'Operating Model'!E8</f>
         <v/>
       </c>
-      <c r="F23" s="23">
+      <c r="F23" s="24">
         <f>F21/'Operating Model'!F8</f>
         <v/>
       </c>
-      <c r="G23" s="23">
+      <c r="G23" s="24">
         <f>G21/'Operating Model'!G8</f>
         <v/>
       </c>
     </row>
+    <row r="25" ht="12" customHeight="1">
+      <c r="B25" s="15" t="inlineStr">
+        <is>
+          <t>Francisco Rodriguez  |  Financial Modeling Portfolio  |  github.com/Azyo1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A19:G19"/>
+    <mergeCell ref="B25:G25"/>
     <mergeCell ref="A12:G12"/>
     <mergeCell ref="A4:G4"/>
   </mergeCells>
@@ -2575,7 +2616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2583,7 +2624,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="29" t="inlineStr">
+      <c r="A1" s="30" t="inlineStr">
         <is>
           <t>Dick's Sporting Goods — Returns Analysis</t>
         </is>
@@ -2597,67 +2638,67 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="15" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>Exit Year EBITDA ($M)</t>
         </is>
       </c>
-      <c r="B4" s="31">
+      <c r="B4" s="32">
         <f>'Operating Model'!G8</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Exit EV / EBITDA Multiple</t>
         </is>
       </c>
-      <c r="B5" s="35">
+      <c r="B5" s="36">
         <f>'Assumptions'!B45</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>Exit Enterprise Value ($M)</t>
         </is>
       </c>
-      <c r="B6" s="19">
+      <c r="B6" s="20">
         <f>B4*B5</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>Less: Net Debt at Exit ($M)</t>
         </is>
       </c>
-      <c r="B7" s="31">
+      <c r="B7" s="32">
         <f>'Debt Schedule'!G8</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>Less: Exit Transaction Fees ($M)</t>
         </is>
       </c>
-      <c r="B8" s="19">
+      <c r="B8" s="20">
         <f>B6*'Assumptions'!B46</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="22" t="inlineStr">
         <is>
           <t>Equity Value to Sponsor ($M)</t>
         </is>
       </c>
-      <c r="B9" s="22">
+      <c r="B9" s="23">
         <f>B6-B7-B8</f>
         <v/>
       </c>
@@ -2670,73 +2711,81 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>Initial Equity Investment ($M)</t>
         </is>
       </c>
-      <c r="B12" s="31">
+      <c r="B12" s="32">
         <f>'Assumptions'!B21</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>Equity Proceeds ($M)</t>
         </is>
       </c>
-      <c r="B13" s="19">
+      <c r="B13" s="20">
         <f>B9</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="22" t="inlineStr">
         <is>
           <t>Multiple of Invested Capital (MOIC)</t>
         </is>
       </c>
-      <c r="B15" s="36">
+      <c r="B15" s="37">
         <f>B13/B12</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="15" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>Hold Period (Years)</t>
         </is>
       </c>
-      <c r="B16" s="37">
+      <c r="B16" s="38">
         <f>'Assumptions'!B44</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A17" s="22" t="inlineStr">
         <is>
           <t>IRR (Approximate)</t>
         </is>
       </c>
-      <c r="B17" s="38">
+      <c r="B17" s="39">
         <f>(B13/B12)^(1/B16)-1</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="15" t="inlineStr">
+      <c r="A18" s="16" t="inlineStr">
         <is>
           <t>Cash-on-Cash Return (MOIC)</t>
         </is>
       </c>
-      <c r="B18" s="23">
+      <c r="B18" s="24">
         <f>B15</f>
         <v/>
       </c>
     </row>
+    <row r="20" ht="12" customHeight="1">
+      <c r="B20" s="15" t="inlineStr">
+        <is>
+          <t>Francisco Rodriguez  |  Financial Modeling Portfolio  |  github.com/Azyo1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
+    <mergeCell ref="B20:C20"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A11:B11"/>
   </mergeCells>
@@ -2751,7 +2800,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2764,7 +2813,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="29" t="inlineStr">
+      <c r="A1" s="30" t="inlineStr">
         <is>
           <t>Dick's Sporting Goods — Sensitivity Analysis</t>
         </is>
@@ -2778,174 +2827,174 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="27" t="inlineStr">
+      <c r="A4" s="28" t="inlineStr">
         <is>
           <t>Entry \ Exit</t>
         </is>
       </c>
-      <c r="B4" s="27" t="inlineStr">
+      <c r="B4" s="28" t="inlineStr">
         <is>
           <t>7.0x</t>
         </is>
       </c>
-      <c r="C4" s="27" t="inlineStr">
+      <c r="C4" s="28" t="inlineStr">
         <is>
           <t>8.0x</t>
         </is>
       </c>
-      <c r="D4" s="27" t="inlineStr">
+      <c r="D4" s="28" t="inlineStr">
         <is>
           <t>9.0x</t>
         </is>
       </c>
-      <c r="E4" s="27" t="inlineStr">
+      <c r="E4" s="28" t="inlineStr">
         <is>
           <t>10.0x</t>
         </is>
       </c>
-      <c r="F4" s="27" t="inlineStr">
+      <c r="F4" s="28" t="inlineStr">
         <is>
           <t>11.0x</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="28" t="inlineStr">
         <is>
           <t>7.0x</t>
         </is>
       </c>
-      <c r="B5" s="39">
+      <c r="B5" s="40">
         <f>IFERROR(((7.0*'Operating Model'!G8-'Debt Schedule'!G8-7.0*'Operating Model'!G8*'Assumptions'!B46)/(7.0*'Assumptions'!B5-'Assumptions'!B9-7.0*'Assumptions'!B5*'Assumptions'!B11))^(1/'Assumptions'!B44)-1,"N/A")</f>
         <v/>
       </c>
-      <c r="C5" s="39">
+      <c r="C5" s="40">
         <f>IFERROR(((8.0*'Operating Model'!G8-'Debt Schedule'!G8-8.0*'Operating Model'!G8*'Assumptions'!B46)/(7.0*'Assumptions'!B5-'Assumptions'!B9-7.0*'Assumptions'!B5*'Assumptions'!B11))^(1/'Assumptions'!B44)-1,"N/A")</f>
         <v/>
       </c>
-      <c r="D5" s="39">
+      <c r="D5" s="40">
         <f>IFERROR(((9.0*'Operating Model'!G8-'Debt Schedule'!G8-9.0*'Operating Model'!G8*'Assumptions'!B46)/(7.0*'Assumptions'!B5-'Assumptions'!B9-7.0*'Assumptions'!B5*'Assumptions'!B11))^(1/'Assumptions'!B44)-1,"N/A")</f>
         <v/>
       </c>
-      <c r="E5" s="39">
+      <c r="E5" s="40">
         <f>IFERROR(((10.0*'Operating Model'!G8-'Debt Schedule'!G8-10.0*'Operating Model'!G8*'Assumptions'!B46)/(7.0*'Assumptions'!B5-'Assumptions'!B9-7.0*'Assumptions'!B5*'Assumptions'!B11))^(1/'Assumptions'!B44)-1,"N/A")</f>
         <v/>
       </c>
-      <c r="F5" s="39">
+      <c r="F5" s="40">
         <f>IFERROR(((11.0*'Operating Model'!G8-'Debt Schedule'!G8-11.0*'Operating Model'!G8*'Assumptions'!B46)/(7.0*'Assumptions'!B5-'Assumptions'!B9-7.0*'Assumptions'!B5*'Assumptions'!B11))^(1/'Assumptions'!B44)-1,"N/A")</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="27" t="inlineStr">
+      <c r="A6" s="28" t="inlineStr">
         <is>
           <t>8.0x</t>
         </is>
       </c>
-      <c r="B6" s="39">
+      <c r="B6" s="40">
         <f>IFERROR(((7.0*'Operating Model'!G8-'Debt Schedule'!G8-7.0*'Operating Model'!G8*'Assumptions'!B46)/(8.0*'Assumptions'!B5-'Assumptions'!B9-8.0*'Assumptions'!B5*'Assumptions'!B11))^(1/'Assumptions'!B44)-1,"N/A")</f>
         <v/>
       </c>
-      <c r="C6" s="39">
+      <c r="C6" s="40">
         <f>IFERROR(((8.0*'Operating Model'!G8-'Debt Schedule'!G8-8.0*'Operating Model'!G8*'Assumptions'!B46)/(8.0*'Assumptions'!B5-'Assumptions'!B9-8.0*'Assumptions'!B5*'Assumptions'!B11))^(1/'Assumptions'!B44)-1,"N/A")</f>
         <v/>
       </c>
-      <c r="D6" s="39">
+      <c r="D6" s="40">
         <f>IFERROR(((9.0*'Operating Model'!G8-'Debt Schedule'!G8-9.0*'Operating Model'!G8*'Assumptions'!B46)/(8.0*'Assumptions'!B5-'Assumptions'!B9-8.0*'Assumptions'!B5*'Assumptions'!B11))^(1/'Assumptions'!B44)-1,"N/A")</f>
         <v/>
       </c>
-      <c r="E6" s="39">
+      <c r="E6" s="40">
         <f>IFERROR(((10.0*'Operating Model'!G8-'Debt Schedule'!G8-10.0*'Operating Model'!G8*'Assumptions'!B46)/(8.0*'Assumptions'!B5-'Assumptions'!B9-8.0*'Assumptions'!B5*'Assumptions'!B11))^(1/'Assumptions'!B44)-1,"N/A")</f>
         <v/>
       </c>
-      <c r="F6" s="39">
+      <c r="F6" s="40">
         <f>IFERROR(((11.0*'Operating Model'!G8-'Debt Schedule'!G8-11.0*'Operating Model'!G8*'Assumptions'!B46)/(8.0*'Assumptions'!B5-'Assumptions'!B9-8.0*'Assumptions'!B5*'Assumptions'!B11))^(1/'Assumptions'!B44)-1,"N/A")</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="27" t="inlineStr">
+      <c r="A7" s="28" t="inlineStr">
         <is>
           <t>9.0x</t>
         </is>
       </c>
-      <c r="B7" s="39">
+      <c r="B7" s="40">
         <f>IFERROR(((7.0*'Operating Model'!G8-'Debt Schedule'!G8-7.0*'Operating Model'!G8*'Assumptions'!B46)/(9.0*'Assumptions'!B5-'Assumptions'!B9-9.0*'Assumptions'!B5*'Assumptions'!B11))^(1/'Assumptions'!B44)-1,"N/A")</f>
         <v/>
       </c>
-      <c r="C7" s="39">
+      <c r="C7" s="40">
         <f>IFERROR(((8.0*'Operating Model'!G8-'Debt Schedule'!G8-8.0*'Operating Model'!G8*'Assumptions'!B46)/(9.0*'Assumptions'!B5-'Assumptions'!B9-9.0*'Assumptions'!B5*'Assumptions'!B11))^(1/'Assumptions'!B44)-1,"N/A")</f>
         <v/>
       </c>
-      <c r="D7" s="40">
+      <c r="D7" s="41">
         <f>IFERROR(((9.0*'Operating Model'!G8-'Debt Schedule'!G8-9.0*'Operating Model'!G8*'Assumptions'!B46)/(9.0*'Assumptions'!B5-'Assumptions'!B9-9.0*'Assumptions'!B5*'Assumptions'!B11))^(1/'Assumptions'!B44)-1,"N/A")</f>
         <v/>
       </c>
-      <c r="E7" s="39">
+      <c r="E7" s="40">
         <f>IFERROR(((10.0*'Operating Model'!G8-'Debt Schedule'!G8-10.0*'Operating Model'!G8*'Assumptions'!B46)/(9.0*'Assumptions'!B5-'Assumptions'!B9-9.0*'Assumptions'!B5*'Assumptions'!B11))^(1/'Assumptions'!B44)-1,"N/A")</f>
         <v/>
       </c>
-      <c r="F7" s="39">
+      <c r="F7" s="40">
         <f>IFERROR(((11.0*'Operating Model'!G8-'Debt Schedule'!G8-11.0*'Operating Model'!G8*'Assumptions'!B46)/(9.0*'Assumptions'!B5-'Assumptions'!B9-9.0*'Assumptions'!B5*'Assumptions'!B11))^(1/'Assumptions'!B44)-1,"N/A")</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="27" t="inlineStr">
+      <c r="A8" s="28" t="inlineStr">
         <is>
           <t>10.0x</t>
         </is>
       </c>
-      <c r="B8" s="39">
+      <c r="B8" s="40">
         <f>IFERROR(((7.0*'Operating Model'!G8-'Debt Schedule'!G8-7.0*'Operating Model'!G8*'Assumptions'!B46)/(10.0*'Assumptions'!B5-'Assumptions'!B9-10.0*'Assumptions'!B5*'Assumptions'!B11))^(1/'Assumptions'!B44)-1,"N/A")</f>
         <v/>
       </c>
-      <c r="C8" s="39">
+      <c r="C8" s="40">
         <f>IFERROR(((8.0*'Operating Model'!G8-'Debt Schedule'!G8-8.0*'Operating Model'!G8*'Assumptions'!B46)/(10.0*'Assumptions'!B5-'Assumptions'!B9-10.0*'Assumptions'!B5*'Assumptions'!B11))^(1/'Assumptions'!B44)-1,"N/A")</f>
         <v/>
       </c>
-      <c r="D8" s="39">
+      <c r="D8" s="40">
         <f>IFERROR(((9.0*'Operating Model'!G8-'Debt Schedule'!G8-9.0*'Operating Model'!G8*'Assumptions'!B46)/(10.0*'Assumptions'!B5-'Assumptions'!B9-10.0*'Assumptions'!B5*'Assumptions'!B11))^(1/'Assumptions'!B44)-1,"N/A")</f>
         <v/>
       </c>
-      <c r="E8" s="39">
+      <c r="E8" s="40">
         <f>IFERROR(((10.0*'Operating Model'!G8-'Debt Schedule'!G8-10.0*'Operating Model'!G8*'Assumptions'!B46)/(10.0*'Assumptions'!B5-'Assumptions'!B9-10.0*'Assumptions'!B5*'Assumptions'!B11))^(1/'Assumptions'!B44)-1,"N/A")</f>
         <v/>
       </c>
-      <c r="F8" s="39">
+      <c r="F8" s="40">
         <f>IFERROR(((11.0*'Operating Model'!G8-'Debt Schedule'!G8-11.0*'Operating Model'!G8*'Assumptions'!B46)/(10.0*'Assumptions'!B5-'Assumptions'!B9-10.0*'Assumptions'!B5*'Assumptions'!B11))^(1/'Assumptions'!B44)-1,"N/A")</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="27" t="inlineStr">
+      <c r="A9" s="28" t="inlineStr">
         <is>
           <t>11.0x</t>
         </is>
       </c>
-      <c r="B9" s="39">
+      <c r="B9" s="40">
         <f>IFERROR(((7.0*'Operating Model'!G8-'Debt Schedule'!G8-7.0*'Operating Model'!G8*'Assumptions'!B46)/(11.0*'Assumptions'!B5-'Assumptions'!B9-11.0*'Assumptions'!B5*'Assumptions'!B11))^(1/'Assumptions'!B44)-1,"N/A")</f>
         <v/>
       </c>
-      <c r="C9" s="39">
+      <c r="C9" s="40">
         <f>IFERROR(((8.0*'Operating Model'!G8-'Debt Schedule'!G8-8.0*'Operating Model'!G8*'Assumptions'!B46)/(11.0*'Assumptions'!B5-'Assumptions'!B9-11.0*'Assumptions'!B5*'Assumptions'!B11))^(1/'Assumptions'!B44)-1,"N/A")</f>
         <v/>
       </c>
-      <c r="D9" s="39">
+      <c r="D9" s="40">
         <f>IFERROR(((9.0*'Operating Model'!G8-'Debt Schedule'!G8-9.0*'Operating Model'!G8*'Assumptions'!B46)/(11.0*'Assumptions'!B5-'Assumptions'!B9-11.0*'Assumptions'!B5*'Assumptions'!B11))^(1/'Assumptions'!B44)-1,"N/A")</f>
         <v/>
       </c>
-      <c r="E9" s="39">
+      <c r="E9" s="40">
         <f>IFERROR(((10.0*'Operating Model'!G8-'Debt Schedule'!G8-10.0*'Operating Model'!G8*'Assumptions'!B46)/(11.0*'Assumptions'!B5-'Assumptions'!B9-11.0*'Assumptions'!B5*'Assumptions'!B11))^(1/'Assumptions'!B44)-1,"N/A")</f>
         <v/>
       </c>
-      <c r="F9" s="39">
+      <c r="F9" s="40">
         <f>IFERROR(((11.0*'Operating Model'!G8-'Debt Schedule'!G8-11.0*'Operating Model'!G8*'Assumptions'!B46)/(11.0*'Assumptions'!B5-'Assumptions'!B9-11.0*'Assumptions'!B5*'Assumptions'!B11))^(1/'Assumptions'!B44)-1,"N/A")</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="41" t="inlineStr">
+      <c r="A11" s="42" t="inlineStr">
         <is>
           <t>Rows = Entry EV/EBITDA Multiple | Columns = Exit EV/EBITDA Multiple</t>
         </is>
@@ -2959,183 +3008,191 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="27" t="inlineStr">
+      <c r="A14" s="28" t="inlineStr">
         <is>
           <t>Entry \ Exit</t>
         </is>
       </c>
-      <c r="B14" s="27" t="inlineStr">
+      <c r="B14" s="28" t="inlineStr">
         <is>
           <t>7.0x</t>
         </is>
       </c>
-      <c r="C14" s="27" t="inlineStr">
+      <c r="C14" s="28" t="inlineStr">
         <is>
           <t>8.0x</t>
         </is>
       </c>
-      <c r="D14" s="27" t="inlineStr">
+      <c r="D14" s="28" t="inlineStr">
         <is>
           <t>9.0x</t>
         </is>
       </c>
-      <c r="E14" s="27" t="inlineStr">
+      <c r="E14" s="28" t="inlineStr">
         <is>
           <t>10.0x</t>
         </is>
       </c>
-      <c r="F14" s="27" t="inlineStr">
+      <c r="F14" s="28" t="inlineStr">
         <is>
           <t>11.0x</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="27" t="inlineStr">
+      <c r="A15" s="28" t="inlineStr">
         <is>
           <t>7.0x</t>
         </is>
       </c>
-      <c r="B15" s="42">
+      <c r="B15" s="43">
         <f>IFERROR((7.0*'Operating Model'!G8-'Debt Schedule'!G8-7.0*'Operating Model'!G8*'Assumptions'!B46)/(7.0*'Assumptions'!B5-'Assumptions'!B9-7.0*'Assumptions'!B5*'Assumptions'!B11),"N/A")</f>
         <v/>
       </c>
-      <c r="C15" s="42">
+      <c r="C15" s="43">
         <f>IFERROR((8.0*'Operating Model'!G8-'Debt Schedule'!G8-8.0*'Operating Model'!G8*'Assumptions'!B46)/(7.0*'Assumptions'!B5-'Assumptions'!B9-7.0*'Assumptions'!B5*'Assumptions'!B11),"N/A")</f>
         <v/>
       </c>
-      <c r="D15" s="42">
+      <c r="D15" s="43">
         <f>IFERROR((9.0*'Operating Model'!G8-'Debt Schedule'!G8-9.0*'Operating Model'!G8*'Assumptions'!B46)/(7.0*'Assumptions'!B5-'Assumptions'!B9-7.0*'Assumptions'!B5*'Assumptions'!B11),"N/A")</f>
         <v/>
       </c>
-      <c r="E15" s="42">
+      <c r="E15" s="43">
         <f>IFERROR((10.0*'Operating Model'!G8-'Debt Schedule'!G8-10.0*'Operating Model'!G8*'Assumptions'!B46)/(7.0*'Assumptions'!B5-'Assumptions'!B9-7.0*'Assumptions'!B5*'Assumptions'!B11),"N/A")</f>
         <v/>
       </c>
-      <c r="F15" s="42">
+      <c r="F15" s="43">
         <f>IFERROR((11.0*'Operating Model'!G8-'Debt Schedule'!G8-11.0*'Operating Model'!G8*'Assumptions'!B46)/(7.0*'Assumptions'!B5-'Assumptions'!B9-7.0*'Assumptions'!B5*'Assumptions'!B11),"N/A")</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="27" t="inlineStr">
+      <c r="A16" s="28" t="inlineStr">
         <is>
           <t>8.0x</t>
         </is>
       </c>
-      <c r="B16" s="42">
+      <c r="B16" s="43">
         <f>IFERROR((7.0*'Operating Model'!G8-'Debt Schedule'!G8-7.0*'Operating Model'!G8*'Assumptions'!B46)/(8.0*'Assumptions'!B5-'Assumptions'!B9-8.0*'Assumptions'!B5*'Assumptions'!B11),"N/A")</f>
         <v/>
       </c>
-      <c r="C16" s="42">
+      <c r="C16" s="43">
         <f>IFERROR((8.0*'Operating Model'!G8-'Debt Schedule'!G8-8.0*'Operating Model'!G8*'Assumptions'!B46)/(8.0*'Assumptions'!B5-'Assumptions'!B9-8.0*'Assumptions'!B5*'Assumptions'!B11),"N/A")</f>
         <v/>
       </c>
-      <c r="D16" s="42">
+      <c r="D16" s="43">
         <f>IFERROR((9.0*'Operating Model'!G8-'Debt Schedule'!G8-9.0*'Operating Model'!G8*'Assumptions'!B46)/(8.0*'Assumptions'!B5-'Assumptions'!B9-8.0*'Assumptions'!B5*'Assumptions'!B11),"N/A")</f>
         <v/>
       </c>
-      <c r="E16" s="42">
+      <c r="E16" s="43">
         <f>IFERROR((10.0*'Operating Model'!G8-'Debt Schedule'!G8-10.0*'Operating Model'!G8*'Assumptions'!B46)/(8.0*'Assumptions'!B5-'Assumptions'!B9-8.0*'Assumptions'!B5*'Assumptions'!B11),"N/A")</f>
         <v/>
       </c>
-      <c r="F16" s="42">
+      <c r="F16" s="43">
         <f>IFERROR((11.0*'Operating Model'!G8-'Debt Schedule'!G8-11.0*'Operating Model'!G8*'Assumptions'!B46)/(8.0*'Assumptions'!B5-'Assumptions'!B9-8.0*'Assumptions'!B5*'Assumptions'!B11),"N/A")</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="27" t="inlineStr">
+      <c r="A17" s="28" t="inlineStr">
         <is>
           <t>9.0x</t>
         </is>
       </c>
-      <c r="B17" s="42">
+      <c r="B17" s="43">
         <f>IFERROR((7.0*'Operating Model'!G8-'Debt Schedule'!G8-7.0*'Operating Model'!G8*'Assumptions'!B46)/(9.0*'Assumptions'!B5-'Assumptions'!B9-9.0*'Assumptions'!B5*'Assumptions'!B11),"N/A")</f>
         <v/>
       </c>
-      <c r="C17" s="42">
+      <c r="C17" s="43">
         <f>IFERROR((8.0*'Operating Model'!G8-'Debt Schedule'!G8-8.0*'Operating Model'!G8*'Assumptions'!B46)/(9.0*'Assumptions'!B5-'Assumptions'!B9-9.0*'Assumptions'!B5*'Assumptions'!B11),"N/A")</f>
         <v/>
       </c>
-      <c r="D17" s="43">
+      <c r="D17" s="44">
         <f>IFERROR((9.0*'Operating Model'!G8-'Debt Schedule'!G8-9.0*'Operating Model'!G8*'Assumptions'!B46)/(9.0*'Assumptions'!B5-'Assumptions'!B9-9.0*'Assumptions'!B5*'Assumptions'!B11),"N/A")</f>
         <v/>
       </c>
-      <c r="E17" s="42">
+      <c r="E17" s="43">
         <f>IFERROR((10.0*'Operating Model'!G8-'Debt Schedule'!G8-10.0*'Operating Model'!G8*'Assumptions'!B46)/(9.0*'Assumptions'!B5-'Assumptions'!B9-9.0*'Assumptions'!B5*'Assumptions'!B11),"N/A")</f>
         <v/>
       </c>
-      <c r="F17" s="42">
+      <c r="F17" s="43">
         <f>IFERROR((11.0*'Operating Model'!G8-'Debt Schedule'!G8-11.0*'Operating Model'!G8*'Assumptions'!B46)/(9.0*'Assumptions'!B5-'Assumptions'!B9-9.0*'Assumptions'!B5*'Assumptions'!B11),"N/A")</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="27" t="inlineStr">
+      <c r="A18" s="28" t="inlineStr">
         <is>
           <t>10.0x</t>
         </is>
       </c>
-      <c r="B18" s="42">
+      <c r="B18" s="43">
         <f>IFERROR((7.0*'Operating Model'!G8-'Debt Schedule'!G8-7.0*'Operating Model'!G8*'Assumptions'!B46)/(10.0*'Assumptions'!B5-'Assumptions'!B9-10.0*'Assumptions'!B5*'Assumptions'!B11),"N/A")</f>
         <v/>
       </c>
-      <c r="C18" s="42">
+      <c r="C18" s="43">
         <f>IFERROR((8.0*'Operating Model'!G8-'Debt Schedule'!G8-8.0*'Operating Model'!G8*'Assumptions'!B46)/(10.0*'Assumptions'!B5-'Assumptions'!B9-10.0*'Assumptions'!B5*'Assumptions'!B11),"N/A")</f>
         <v/>
       </c>
-      <c r="D18" s="42">
+      <c r="D18" s="43">
         <f>IFERROR((9.0*'Operating Model'!G8-'Debt Schedule'!G8-9.0*'Operating Model'!G8*'Assumptions'!B46)/(10.0*'Assumptions'!B5-'Assumptions'!B9-10.0*'Assumptions'!B5*'Assumptions'!B11),"N/A")</f>
         <v/>
       </c>
-      <c r="E18" s="42">
+      <c r="E18" s="43">
         <f>IFERROR((10.0*'Operating Model'!G8-'Debt Schedule'!G8-10.0*'Operating Model'!G8*'Assumptions'!B46)/(10.0*'Assumptions'!B5-'Assumptions'!B9-10.0*'Assumptions'!B5*'Assumptions'!B11),"N/A")</f>
         <v/>
       </c>
-      <c r="F18" s="42">
+      <c r="F18" s="43">
         <f>IFERROR((11.0*'Operating Model'!G8-'Debt Schedule'!G8-11.0*'Operating Model'!G8*'Assumptions'!B46)/(10.0*'Assumptions'!B5-'Assumptions'!B9-10.0*'Assumptions'!B5*'Assumptions'!B11),"N/A")</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="27" t="inlineStr">
+      <c r="A19" s="28" t="inlineStr">
         <is>
           <t>11.0x</t>
         </is>
       </c>
-      <c r="B19" s="42">
+      <c r="B19" s="43">
         <f>IFERROR((7.0*'Operating Model'!G8-'Debt Schedule'!G8-7.0*'Operating Model'!G8*'Assumptions'!B46)/(11.0*'Assumptions'!B5-'Assumptions'!B9-11.0*'Assumptions'!B5*'Assumptions'!B11),"N/A")</f>
         <v/>
       </c>
-      <c r="C19" s="42">
+      <c r="C19" s="43">
         <f>IFERROR((8.0*'Operating Model'!G8-'Debt Schedule'!G8-8.0*'Operating Model'!G8*'Assumptions'!B46)/(11.0*'Assumptions'!B5-'Assumptions'!B9-11.0*'Assumptions'!B5*'Assumptions'!B11),"N/A")</f>
         <v/>
       </c>
-      <c r="D19" s="42">
+      <c r="D19" s="43">
         <f>IFERROR((9.0*'Operating Model'!G8-'Debt Schedule'!G8-9.0*'Operating Model'!G8*'Assumptions'!B46)/(11.0*'Assumptions'!B5-'Assumptions'!B9-11.0*'Assumptions'!B5*'Assumptions'!B11),"N/A")</f>
         <v/>
       </c>
-      <c r="E19" s="42">
+      <c r="E19" s="43">
         <f>IFERROR((10.0*'Operating Model'!G8-'Debt Schedule'!G8-10.0*'Operating Model'!G8*'Assumptions'!B46)/(11.0*'Assumptions'!B5-'Assumptions'!B9-11.0*'Assumptions'!B5*'Assumptions'!B11),"N/A")</f>
         <v/>
       </c>
-      <c r="F19" s="42">
+      <c r="F19" s="43">
         <f>IFERROR((11.0*'Operating Model'!G8-'Debt Schedule'!G8-11.0*'Operating Model'!G8*'Assumptions'!B46)/(11.0*'Assumptions'!B5-'Assumptions'!B9-11.0*'Assumptions'!B5*'Assumptions'!B11),"N/A")</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="41" t="inlineStr">
+      <c r="A21" s="42" t="inlineStr">
         <is>
           <t>Rows = Entry EV/EBITDA Multiple | Columns = Exit EV/EBITDA Multiple</t>
         </is>
       </c>
     </row>
+    <row r="23" ht="12" customHeight="1">
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>Francisco Rodriguez  |  Financial Modeling Portfolio  |  github.com/Azyo1</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A13:F13"/>
+    <mergeCell ref="B23:G23"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:F9">
     <cfRule type="colorScale" priority="1">

</xml_diff>